<commit_message>
Add runbooks for Payobook SaaS platform operations
- Introduced SAAS_RESIZE_RUNBOOK.md detailing the manual process for resizing the Payobook platform machine, including pre- and post-resize steps, expected downtime, and verification checks.
- Created SAAS_RUNBOOK.md as a comprehensive operational reference for the multi-tenant Payobook platform, covering architecture, go-live procedures, golden template rebuilds, code deployment rituals, known issues, and tenant management.
</commit_message>
<xml_diff>
--- a/Migration/Price_List_Adjustments_Rules_20250917 V3.2 Scrubbed.xlsx
+++ b/Migration/Price_List_Adjustments_Rules_20250917 V3.2 Scrubbed.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adity/Documents/GitHub/health19/Migration/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2A357EF-5A2A-2649-BB9F-5821D7F7A2F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="20" windowWidth="16100" windowHeight="9660"/>
+    <workbookView xWindow="140" yWindow="660" windowWidth="38080" windowHeight="20800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hanoi_Adjustments_Clean" sheetId="1" r:id="rId1"/>
@@ -12,7 +18,20 @@
     <sheet name="Hanoi_Base_Clean_v3" sheetId="3" r:id="rId3"/>
     <sheet name="HCMC_Base_Clean_v3" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -814,7 +833,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -867,12 +886,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -883,14 +901,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -928,7 +949,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1000,7 +1021,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1173,23 +1194,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="49.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="49.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="48.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="34.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="48.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1221,7 +1242,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1253,7 +1274,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1285,7 +1306,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1317,7 +1338,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1349,7 +1370,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1381,7 +1402,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1413,7 +1434,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1445,7 +1466,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1477,7 +1498,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1509,7 +1530,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1541,7 +1562,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1573,7 +1594,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1605,7 +1626,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1637,7 +1658,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -1669,7 +1690,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -1701,7 +1722,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -1733,7 +1754,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -1765,7 +1786,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -1797,7 +1818,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -1829,7 +1850,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -1861,7 +1882,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -1893,7 +1914,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -1922,7 +1943,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -1954,7 +1975,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>10</v>
       </c>
@@ -1986,7 +2007,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>10</v>
       </c>
@@ -2018,7 +2039,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -2047,7 +2068,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>10</v>
       </c>
@@ -2079,7 +2100,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>10</v>
       </c>
@@ -2108,7 +2129,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>10</v>
       </c>
@@ -2140,7 +2161,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>10</v>
       </c>
@@ -2169,7 +2190,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -2198,7 +2219,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>10</v>
       </c>
@@ -2230,7 +2251,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>10</v>
       </c>
@@ -2262,7 +2283,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>10</v>
       </c>
@@ -2300,23 +2321,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J72"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="64" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="48.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="48.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="48.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="48.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2348,7 +2369,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>98</v>
       </c>
@@ -2380,7 +2401,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>98</v>
       </c>
@@ -2412,7 +2433,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>98</v>
       </c>
@@ -2444,7 +2465,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>98</v>
       </c>
@@ -2476,7 +2497,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>98</v>
       </c>
@@ -2508,7 +2529,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>98</v>
       </c>
@@ -2540,7 +2561,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>98</v>
       </c>
@@ -2572,7 +2593,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>98</v>
       </c>
@@ -2604,7 +2625,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>98</v>
       </c>
@@ -2636,7 +2657,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>98</v>
       </c>
@@ -2668,7 +2689,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>98</v>
       </c>
@@ -2700,7 +2721,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>98</v>
       </c>
@@ -2732,7 +2753,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>98</v>
       </c>
@@ -2764,7 +2785,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>98</v>
       </c>
@@ -2796,7 +2817,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>98</v>
       </c>
@@ -2828,7 +2849,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>98</v>
       </c>
@@ -2860,7 +2881,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>98</v>
       </c>
@@ -2892,7 +2913,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>98</v>
       </c>
@@ -2924,7 +2945,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>98</v>
       </c>
@@ -2956,7 +2977,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>98</v>
       </c>
@@ -2988,7 +3009,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>98</v>
       </c>
@@ -3020,7 +3041,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>98</v>
       </c>
@@ -3052,7 +3073,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>98</v>
       </c>
@@ -3084,7 +3105,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>98</v>
       </c>
@@ -3116,7 +3137,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>98</v>
       </c>
@@ -3148,7 +3169,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>98</v>
       </c>
@@ -3180,7 +3201,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>98</v>
       </c>
@@ -3212,7 +3233,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>98</v>
       </c>
@@ -3244,7 +3265,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>98</v>
       </c>
@@ -3276,7 +3297,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>98</v>
       </c>
@@ -3308,7 +3329,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>98</v>
       </c>
@@ -3340,7 +3361,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>98</v>
       </c>
@@ -3372,7 +3393,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>98</v>
       </c>
@@ -3404,7 +3425,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>98</v>
       </c>
@@ -3436,7 +3457,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>98</v>
       </c>
@@ -3468,7 +3489,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>98</v>
       </c>
@@ -3500,7 +3521,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>98</v>
       </c>
@@ -3532,7 +3553,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>98</v>
       </c>
@@ -3564,7 +3585,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>98</v>
       </c>
@@ -3596,7 +3617,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>98</v>
       </c>
@@ -3628,7 +3649,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>98</v>
       </c>
@@ -3660,7 +3681,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>98</v>
       </c>
@@ -3692,7 +3713,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>98</v>
       </c>
@@ -3724,7 +3745,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>98</v>
       </c>
@@ -3756,7 +3777,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>98</v>
       </c>
@@ -3788,7 +3809,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>98</v>
       </c>
@@ -3820,7 +3841,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>98</v>
       </c>
@@ -3852,7 +3873,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>98</v>
       </c>
@@ -3884,7 +3905,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>98</v>
       </c>
@@ -3916,7 +3937,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>98</v>
       </c>
@@ -3948,7 +3969,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>98</v>
       </c>
@@ -3980,7 +4001,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>98</v>
       </c>
@@ -4012,7 +4033,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>98</v>
       </c>
@@ -4044,7 +4065,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -4076,7 +4097,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>98</v>
       </c>
@@ -4108,7 +4129,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>98</v>
       </c>
@@ -4140,7 +4161,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>98</v>
       </c>
@@ -4172,7 +4193,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>98</v>
       </c>
@@ -4204,7 +4225,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>98</v>
       </c>
@@ -4236,7 +4257,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>98</v>
       </c>
@@ -4268,7 +4289,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>98</v>
       </c>
@@ -4300,7 +4321,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>98</v>
       </c>
@@ -4332,7 +4353,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>98</v>
       </c>
@@ -4364,7 +4385,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>98</v>
       </c>
@@ -4396,7 +4417,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>98</v>
       </c>
@@ -4425,7 +4446,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>98</v>
       </c>
@@ -4454,7 +4475,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>98</v>
       </c>
@@ -4486,7 +4507,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>98</v>
       </c>
@@ -4518,7 +4539,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>98</v>
       </c>
@@ -4550,7 +4571,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>98</v>
       </c>
@@ -4579,7 +4600,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>98</v>
       </c>
@@ -4614,27 +4635,27 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:U39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="53.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.1640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>161</v>
       </c>
@@ -4699,7 +4720,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4746,7 +4767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4793,7 +4814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -4840,7 +4861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4887,7 +4908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4934,7 +4955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -4981,7 +5002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -5028,7 +5049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -5075,7 +5096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -5122,7 +5143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -5169,7 +5190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -5216,7 +5237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -5263,7 +5284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -5310,7 +5331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -5357,7 +5378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -5404,7 +5425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -5451,7 +5472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -5498,7 +5519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -5545,7 +5566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -5592,7 +5613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -5639,7 +5660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -5686,7 +5707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -5733,7 +5754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -5780,7 +5801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -5827,7 +5848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -5874,7 +5895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -5921,7 +5942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -5968,7 +5989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -6015,7 +6036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -6062,7 +6083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -6109,7 +6130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -6156,7 +6177,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -6203,7 +6224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -6250,7 +6271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -6297,7 +6318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -6344,7 +6365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -6391,7 +6412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -6438,7 +6459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -6491,28 +6512,28 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:U44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="54.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="54.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="25.90625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>161</v>
       </c>
@@ -6577,7 +6598,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -6621,7 +6642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -6665,7 +6686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -6709,7 +6730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -6753,7 +6774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -6797,7 +6818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -6841,403 +6862,403 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>200</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" t="s">
         <v>195</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" t="s">
         <v>196</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" t="s">
         <v>197</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" t="s">
         <v>116</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" t="s">
         <v>199</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" t="s">
         <v>199</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8">
         <v>300000</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" t="s">
         <v>188</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="M8" t="s">
         <v>194</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="N8" t="s">
         <v>190</v>
       </c>
-      <c r="O8" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>200</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" t="s">
         <v>195</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" t="s">
         <v>196</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" t="s">
         <v>197</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" t="s">
         <v>117</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" t="s">
         <v>199</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" t="s">
         <v>199</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9">
         <v>300000</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" t="s">
         <v>188</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="M9" t="s">
         <v>194</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="N9" t="s">
         <v>190</v>
       </c>
-      <c r="O9" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>200</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" t="s">
         <v>195</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" t="s">
         <v>196</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" t="s">
         <v>197</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" t="s">
         <v>118</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" t="s">
         <v>199</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" t="s">
         <v>199</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10">
         <v>150000</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" t="s">
         <v>188</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="M10" t="s">
         <v>194</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N10" t="s">
         <v>190</v>
       </c>
-      <c r="O10" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>200</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" t="s">
         <v>195</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" t="s">
         <v>196</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" t="s">
         <v>197</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" t="s">
         <v>39</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" t="s">
         <v>199</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" t="s">
         <v>199</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11">
         <v>150000</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" t="s">
         <v>188</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="M11" t="s">
         <v>194</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="N11" t="s">
         <v>190</v>
       </c>
-      <c r="O11" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>200</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" t="s">
         <v>195</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" t="s">
         <v>196</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" t="s">
         <v>197</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" t="s">
         <v>119</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" t="s">
         <v>199</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="J12" t="s">
         <v>199</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12">
         <v>150000</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="L12" t="s">
         <v>188</v>
       </c>
-      <c r="M12" s="2" t="s">
+      <c r="M12" t="s">
         <v>194</v>
       </c>
-      <c r="N12" s="2" t="s">
+      <c r="N12" t="s">
         <v>190</v>
       </c>
-      <c r="O12" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>200</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" t="s">
         <v>195</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" t="s">
         <v>196</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" t="s">
         <v>197</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" t="s">
         <v>120</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" t="s">
         <v>199</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="J13" t="s">
         <v>199</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13">
         <v>150000</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="L13" t="s">
         <v>188</v>
       </c>
-      <c r="M13" s="2" t="s">
+      <c r="M13" t="s">
         <v>194</v>
       </c>
-      <c r="N13" s="2" t="s">
+      <c r="N13" t="s">
         <v>190</v>
       </c>
-      <c r="O13" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>200</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" t="s">
         <v>195</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" t="s">
         <v>196</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" t="s">
         <v>197</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" t="s">
         <v>121</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I14" t="s">
         <v>199</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="J14" t="s">
         <v>199</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14">
         <v>250000</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="L14" t="s">
         <v>188</v>
       </c>
-      <c r="M14" s="2" t="s">
+      <c r="M14" t="s">
         <v>194</v>
       </c>
-      <c r="N14" s="2" t="s">
+      <c r="N14" t="s">
         <v>190</v>
       </c>
-      <c r="O14" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" t="s">
         <v>200</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" t="s">
         <v>101</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" t="s">
         <v>195</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" t="s">
         <v>196</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" t="s">
         <v>197</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" t="s">
         <v>43</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" t="s">
         <v>199</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>199</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15">
         <v>200000</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="L15" t="s">
         <v>188</v>
       </c>
-      <c r="M15" s="2" t="s">
+      <c r="M15" t="s">
         <v>194</v>
       </c>
-      <c r="N15" s="2" t="s">
+      <c r="N15" t="s">
         <v>190</v>
       </c>
-      <c r="O15" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="O15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" t="s">
         <v>200</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" t="s">
         <v>101</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" t="s">
         <v>195</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" t="s">
         <v>196</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" t="s">
         <v>197</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" t="s">
         <v>247</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" t="s">
         <v>199</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="J16" t="s">
         <v>199</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16">
         <v>200000</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="L16" t="s">
         <v>188</v>
       </c>
-      <c r="M16" s="2" t="s">
+      <c r="M16" t="s">
         <v>194</v>
       </c>
-      <c r="N16" s="2" t="s">
+      <c r="N16" t="s">
         <v>190</v>
       </c>
-      <c r="O16" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="O16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -7281,7 +7302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -7325,7 +7346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -7369,7 +7390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -7413,7 +7434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -7457,7 +7478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -7501,7 +7522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -7545,7 +7566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -7589,7 +7610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -7633,7 +7654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -7677,7 +7698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -7721,7 +7742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -7765,7 +7786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -7809,7 +7830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -7853,7 +7874,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -7897,7 +7918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -7941,7 +7962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -7985,7 +8006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -8029,7 +8050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -8073,7 +8094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -8117,7 +8138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -8161,7 +8182,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -8205,7 +8226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -8249,7 +8270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -8293,7 +8314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -8337,7 +8358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -8381,7 +8402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -8425,7 +8446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>

</xml_diff>